<commit_message>
archivos en la nube lectura por nombre de  hoja completado
</commit_message>
<xml_diff>
--- a/cypress/fixtures/variables.xlsx
+++ b/cypress/fixtures/variables.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="12">
   <si>
     <t>Usuario</t>
   </si>
@@ -25,6 +25,15 @@
     <t>URL_DATOS</t>
   </si>
   <si>
+    <t>Usuario_Auth</t>
+  </si>
+  <si>
+    <t>Password_Auth</t>
+  </si>
+  <si>
+    <t>Motivo_Auth</t>
+  </si>
+  <si>
     <t>OPERADORQA</t>
   </si>
   <si>
@@ -35,6 +44,9 @@
   </si>
   <si>
     <t>https://docs.google.com/spreadsheets/d/1_xriSLIwwVjPl8SPQz6HpPENpfWiztH_Avw6PdiYhY8/export?format=xlsx</t>
+  </si>
+  <si>
+    <t>QA</t>
   </si>
 </sst>
 </file>
@@ -120,7 +132,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -138,16 +150,19 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="right" readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="right" readingOrder="0" vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -367,6 +382,7 @@
     <col customWidth="1" min="3" max="3" width="47.13"/>
     <col customWidth="1" min="4" max="4" width="86.0"/>
     <col customWidth="1" min="5" max="5" width="80.0"/>
+    <col customWidth="1" min="6" max="6" width="12.88"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -382,9 +398,15 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
@@ -400,40 +422,45 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D2" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="4"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="6"/>
-      <c r="J2" s="6"/>
-      <c r="K2" s="6"/>
-      <c r="L2" s="6"/>
-      <c r="M2" s="6"/>
-      <c r="N2" s="6"/>
-      <c r="O2" s="6"/>
-      <c r="P2" s="6"/>
-      <c r="Q2" s="6"/>
-      <c r="R2" s="6"/>
-      <c r="S2" s="6"/>
+      <c r="F2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H2" s="7"/>
+      <c r="I2" s="7"/>
+      <c r="J2" s="7"/>
+      <c r="K2" s="7"/>
+      <c r="L2" s="7"/>
+      <c r="M2" s="7"/>
+      <c r="N2" s="7"/>
+      <c r="O2" s="7"/>
+      <c r="P2" s="7"/>
+      <c r="Q2" s="7"/>
+      <c r="R2" s="7"/>
+      <c r="S2" s="7"/>
     </row>
     <row r="3">
-      <c r="A3" s="7"/>
       <c r="B3" s="8"/>
       <c r="D3" s="9"/>
     </row>
     <row r="4">
-      <c r="A4" s="7"/>
+      <c r="A4" s="10"/>
       <c r="B4" s="8"/>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
cambios en la autorizacion
</commit_message>
<xml_diff>
--- a/cypress/fixtures/variables.xlsx
+++ b/cypress/fixtures/variables.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="18">
   <si>
     <t>Usuario</t>
   </si>
@@ -56,6 +56,15 @@
   </si>
   <si>
     <t>QA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HELMUTES </t>
+  </si>
+  <si>
+    <t>BANCOCCI11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://plataformabocci-prod.bytesw.cloud </t>
   </si>
 </sst>
 </file>
@@ -496,12 +505,24 @@
       <c r="D5" s="9"/>
       <c r="E5" s="9"/>
     </row>
+    <row r="7">
+      <c r="A7" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>17</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
     <hyperlink r:id="rId2" ref="D2"/>
     <hyperlink r:id="rId3" ref="E2"/>
+    <hyperlink r:id="rId4" ref="C7"/>
   </hyperlinks>
-  <drawing r:id="rId4"/>
+  <drawing r:id="rId5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ultimos cambios en plataforma ignorar archivo prod persona natural
</commit_message>
<xml_diff>
--- a/cypress/fixtures/variables.xlsx
+++ b/cypress/fixtures/variables.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="21">
   <si>
     <t>Usuario</t>
   </si>
@@ -43,31 +43,34 @@
     <t>HELMUTES</t>
   </si>
   <si>
-    <t>BANCOCCI11</t>
+    <t>BANCOCCI12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://plataforma2v7-psi.bytesw.cloud/ </t>
+  </si>
+  <si>
+    <t>https://docs.google.com/spreadsheets/d/1_xriSLIwwVjPl8SPQz6HpPENpfWiztH_Avw6PdiYhY8/export?format=xlsx</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/spreadsheets/d/1-woFEZDdXnT4jXsWMXwbzSl-RwaO4XKlup4Klh_GlNc/export?format=xlsx</t>
+  </si>
+  <si>
+    <t>QA</t>
+  </si>
+  <si>
+    <t>Remota</t>
+  </si>
+  <si>
+    <t>adminqa</t>
+  </si>
+  <si>
+    <t>byte25</t>
+  </si>
+  <si>
+    <t>https://plataforma-staging.bytesw.cloud/</t>
   </si>
   <si>
     <t xml:space="preserve">https://plataformabocci-prod.bytesw.cloud </t>
-  </si>
-  <si>
-    <t>https://docs.google.com/spreadsheets/d/1_xriSLIwwVjPl8SPQz6HpPENpfWiztH_Avw6PdiYhY8/export?format=xlsx</t>
-  </si>
-  <si>
-    <t>https://docs.google.com/spreadsheets/d/1-woFEZDdXnT4jXsWMXwbzSl-RwaO4XKlup4Klh_GlNc/export?format=xlsx</t>
-  </si>
-  <si>
-    <t>QA</t>
-  </si>
-  <si>
-    <t>Remota</t>
-  </si>
-  <si>
-    <t>adminqa</t>
-  </si>
-  <si>
-    <t>byte25</t>
-  </si>
-  <si>
-    <t>https://plataforma-staging.bytesw.cloud/</t>
   </si>
   <si>
     <t>/export?format=xlsx</t>
@@ -77,7 +80,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -133,6 +136,10 @@
       <sz val="8.0"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <color rgb="FF0000FF"/>
     </font>
   </fonts>
   <fills count="3">
@@ -169,7 +176,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -208,6 +215,9 @@
       <alignment horizontal="right" readingOrder="0" vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -426,7 +436,8 @@
     <col customWidth="1" min="1" max="1" width="15.63"/>
     <col customWidth="1" min="2" max="2" width="16.38"/>
     <col customWidth="1" min="3" max="3" width="47.13"/>
-    <col customWidth="1" min="4" max="5" width="86.0"/>
+    <col customWidth="1" min="4" max="4" width="86.0"/>
+    <col customWidth="1" min="5" max="5" width="135.13"/>
     <col customWidth="1" min="6" max="6" width="11.5"/>
     <col customWidth="1" min="7" max="7" width="12.88"/>
     <col customWidth="1" min="9" max="9" width="11.75"/>
@@ -494,7 +505,7 @@
       </c>
       <c r="G2" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>BANCOCCI11</v>
+        <v>BANCOCCI12</v>
       </c>
       <c r="H2" s="7" t="s">
         <v>14</v>
@@ -550,15 +561,18 @@
         <v>10</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="13"/>
+      <c r="C10" s="14" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -573,7 +587,8 @@
     <hyperlink r:id="rId3" ref="E2"/>
     <hyperlink r:id="rId4" ref="C6"/>
     <hyperlink r:id="rId5" ref="C8"/>
+    <hyperlink r:id="rId6" ref="C10"/>
   </hyperlinks>
-  <drawing r:id="rId6"/>
+  <drawing r:id="rId7"/>
 </worksheet>
 </file>
</xml_diff>